<commit_message>
Update member and last-updated dates
</commit_message>
<xml_diff>
--- a/about/members.xlsx
+++ b/about/members.xlsx
@@ -2637,12 +2637,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Frances Hadley</t>
+          <t>Daniel Ma</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>franceshadley@fastmail.co.uk</t>
+          <t>danielma4114@gmail.com</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2652,12 +2652,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>University of Edinburgh</t>
+          <t>Alum, Yale University</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2025 ACF Winter Editor</t>
+          <t>2022 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -2666,12 +2666,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Jacky Xu</t>
+          <t>Frances Hadley</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>hx289@cornell.edu</t>
+          <t>franceshadley@fastmail.co.uk</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Cornell University</t>
+          <t>University of Edinburgh</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2695,12 +2695,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>James Wang</t>
+          <t>Jacky Xu</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>jamesjianda@gmail.com</t>
+          <t>hx289@cornell.edu</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2710,12 +2710,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>University of Ottawa</t>
+          <t>Cornell University</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2024 ACF Fall Editor</t>
+          <t>2025 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -2724,12 +2724,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Jamie Burchett</t>
+          <t>James Wang</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>jb4g21@gmail.com</t>
+          <t>jamesjianda@gmail.com</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2739,12 +2739,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>University of Southampton</t>
+          <t>University of Ottawa</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2025 ACF Winter Editor</t>
+          <t>2024 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -2753,12 +2753,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Jason Zhang</t>
+          <t>Jamie Burchett</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>jiajunzhang.jason@gmail.com</t>
+          <t>jb4g21@gmail.com</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>University of Toronto</t>
+          <t>University of Southampton</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2025 ACF Fall Editor</t>
+          <t>2025 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -2782,12 +2782,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Jay Kim</t>
+          <t>Jason Zhang</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>jayk13th@gmail.com</t>
+          <t>jiajunzhang.jason@gmail.com</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2797,12 +2797,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>University of Chicago</t>
+          <t>University of Toronto</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026 ACF Regionals Editor</t>
+          <t>2025 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -2811,12 +2811,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Jeffrey Fung</t>
+          <t>Jay Kim</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>jeffreyfung@college.harvard.edu</t>
+          <t>jayk13th@gmail.com</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2826,12 +2826,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Harvard University</t>
+          <t>University of Chicago</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2023 ACF Fall Editor</t>
+          <t>2026 ACF Regionals Editor</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -2840,12 +2840,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Jeremy Cummings</t>
+          <t>Jeffrey Fung</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>jeremy.cummings476@gmail.com</t>
+          <t>jeffreyfung@college.harvard.edu</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2855,12 +2855,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Alum, Washington University in St. Louis</t>
+          <t>Harvard University</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2025 ACF Regionals Co-Head Editor</t>
+          <t>2023 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -2869,12 +2869,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Joel Miles</t>
+          <t>Jeremy Cummings</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>joel.miles925@gmail.com</t>
+          <t>jeremy.cummings476@gmail.com</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2884,12 +2884,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>University of Minnesota</t>
+          <t>Alum, Washington University in St. Louis</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2023 ACF Winter Editor</t>
+          <t>2025 ACF Regionals Co-Head Editor</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -2898,12 +2898,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Kevin Wang</t>
+          <t>Joel Miles</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>pandasmoothie@gmail.com</t>
+          <t>joel.miles925@gmail.com</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2913,12 +2913,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Alum, Amherst College</t>
+          <t>University of Minnesota</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2024 ACF Nationals Editor</t>
+          <t>2023 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -2927,12 +2927,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Kuleen Sasse</t>
+          <t>Kevin Wang</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>cometku@gmail.com</t>
+          <t>pandasmoothie@gmail.com</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2942,12 +2942,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Johns Hopkins University</t>
+          <t>Alum, Amherst College</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2025 ACF Nationals Assistant Tournament Director</t>
+          <t>2024 ACF Nationals Editor</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -2956,12 +2956,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Linus Luu</t>
+          <t>Kuleen Sasse</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>linusluu22@gmail.com</t>
+          <t>cometku@gmail.com</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2971,12 +2971,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Cambridge University</t>
+          <t>Johns Hopkins University</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2025 ACF Winter Editor</t>
+          <t>2025 ACF Nationals Assistant Tournament Director</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -2985,12 +2985,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Logan Mathis</t>
+          <t>Linus Luu</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>loganmathisloganmathis@gmail.com</t>
+          <t>linusluu22@gmail.com</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2998,10 +2998,14 @@
           <t>provisional</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Cambridge University</t>
+        </is>
+      </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2025 ACF Nationals Assistant Tournament Director</t>
+          <t>2025 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -3010,12 +3014,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Lucia Gellert</t>
+          <t>Logan Mathis</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>luciagellert27@gmail.com</t>
+          <t>loganmathisloganmathis@gmail.com</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3026,7 +3030,7 @@
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2025 ACF Fall Editor</t>
+          <t>2025 ACF Nationals Assistant Tournament Director</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -3035,12 +3039,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Noah Chin</t>
+          <t>Lucia Gellert</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>noahchin05@vt.edu</t>
+          <t>luciagellert27@gmail.com</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3048,11 +3052,7 @@
           <t>provisional</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Virginia Polytechnic Institute and State University</t>
-        </is>
-      </c>
+      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
           <t>2025 ACF Fall Editor</t>
@@ -3064,12 +3064,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Ophelia Cherry-Pulay</t>
+          <t>Noah Chin</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>opheliacherrypulay25@usn.org</t>
+          <t>noahchin05@vt.edu</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3079,12 +3079,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>USN Quizbowl</t>
+          <t>Virginia Polytechnic Institute and State University</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2024 ACF Fall Editor</t>
+          <t>2025 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -3093,53 +3093,57 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>Ophelia Cherry-Pulay</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>opheliacherrypulay25@usn.org</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>USN Quizbowl</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2024 ACF Fall Editor</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>Rhys Lewis</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>rhysglewis14@gmail.com</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>Alum, Cambridge University
 Alum, Sheffield University</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>2025 ACF Fall Editor</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Shourjo Ganguli</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>shourjoganguli2004@gmail.com</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>2023 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -3148,12 +3152,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Sinecio Morales</t>
+          <t>Shourjo Ganguli</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>sineciomoralesqb@gmail.com</t>
+          <t>shourjoganguli2004@gmail.com</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3161,14 +3165,10 @@
           <t>provisional</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Johns Hopkins University</t>
-        </is>
-      </c>
+      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2025 ACF Winter Editor</t>
+          <t>2023 ACF Fall Editor</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -3177,12 +3177,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Sky Li</t>
+          <t>Sinecio Morales</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>skylimail42@gmail.com</t>
+          <t>sineciomoralesqb@gmail.com</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3192,12 +3192,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Ph.D., University of Toronto</t>
+          <t>Johns Hopkins University</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2024 ACF Winter Editor</t>
+          <t>2025 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -3206,10 +3206,14 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Steven Yuan</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr"/>
+          <t>Sky Li</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>skylimail42@gmail.com</t>
+        </is>
+      </c>
       <c r="C91" t="inlineStr">
         <is>
           <t>provisional</t>
@@ -3217,12 +3221,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>University of California, Berkeley</t>
+          <t>Ph.D., University of Toronto</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2025 ACF Winter Editor</t>
+          <t>2024 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -3231,14 +3235,10 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Vincent Du</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>vincent.duyuan@gmail.com</t>
-        </is>
-      </c>
+          <t>Steven Yuan</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>provisional</t>
@@ -3246,12 +3246,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>University of North Carolina, Chapel Hill</t>
+          <t>University of California, Berkeley</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2024 ACF Regionals Editor</t>
+          <t>2025 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -3260,56 +3260,85 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>Vincent Du</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>vincent.duyuan@gmail.com</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>University of North Carolina, Chapel Hill</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>2024 ACF Regionals Editor</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
           <t>Young Fenimore Lee</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>youngflee99@gmail.com</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>Ohio University
 Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>2026 ACF Nationals Assistant Tournament Director</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
         <is>
           <t>Adam Silverman</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>adsilverman627@gmail.com</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
         <is>
           <t>Ph.D., Northwestern University
 Alum, Georgia Tech</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>2013 ACF Fall Editor
 2014 ACF Regionals Editor
@@ -3318,32 +3347,32 @@
 2023 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>Alex Damisch</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>alexandra.damisch@gmail.com</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
         <is>
           <t>M.S., DePaul University
 Alumna, Lawrence University</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>2018-19, Treasurer
 2018 ACF Nationals Logistics
@@ -3353,63 +3382,63 @@
 2020-21, President</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
         <is>
           <t>Andrew Feist</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>tabstopva@gmail.com</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
         <is>
           <t>A.M. and Ph.D., Duke University
 Alum, University of Central Missouri</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="E97" t="inlineStr">
         <is>
           <t>2018 ACF Nationals Stats Director
 2019-19, Treasurer
 2019 ACF Nationals Stats Director</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
         <is>
           <t>Andrew Wang</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>wangandr95@gmail.com</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
         <is>
           <t>Alum, University of Illinois, Urbana-Champaign</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
+      <c r="E98" t="inlineStr">
         <is>
           <t>2015 ACF Fall Editor
 2018 ACF Nationals Editor
@@ -3417,33 +3446,33 @@
 2020 ACF Winter Science Oversight</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t>Andrew Yaphe</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>andrew.yaphe@naqt.com</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
         <is>
           <t>J.D., Stanford University Law School
 University of Chicago
 Alum, University of Virginia</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="E99" t="inlineStr">
         <is>
           <t>2000 ACF Regionals Head Editor
 2001 ACF Nationals Editor
@@ -3454,123 +3483,123 @@
 2007 ACF Nationals Head Editor</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>Annabelle Yang</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>ayang6089@gmail.com</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
         <is>
           <t>MD, Washington University in St. Louis
 Alum, Duke University</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>2021 ACF Regionals Editor
 2022 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
         <is>
           <t>Arjun Nageswaran</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>ArjunFeb1803@gmail.com</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
         <is>
           <t>Harvard University</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>2020 ACF Fall Editor
 2022 ACF Fall Co-Head Editor
 2022 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
         <is>
           <t>Ben Miller</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>benmillerbenmiller@gmail.com</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
         <is>
           <t>Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>2019 ACF Fall Editor
 2020 ACF Fall Head Editor</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
         <is>
           <t>Bernadette Spencer</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>bernadette.spencer@gmail.com</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
         <is>
           <t>Alum, University of Minnesota</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>2017 ACF Nationals Travel Logistics
 2018 ACF Nationals Travel Logistics
@@ -3579,32 +3608,32 @@
 2022 ACF Nationals Travel Logistics</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
         <is>
           <t>Billy Busse</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B104" t="inlineStr">
         <is>
           <t>wtbusse@gmail.com</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
         <is>
           <t>M.D., Rosalind Franklin University
 Alum, University of Illinois, Urbana-Champaign</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E104" t="inlineStr">
         <is>
           <t>2015 ACF Nationals Editor
 2016 ACF Nationals Editor
@@ -3613,124 +3642,124 @@
 2020 ACF Regionals Science Oversight</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
         <is>
           <t>Bruce Arthur</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>boctavianarthur@gmail.com</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
         <is>
           <t>Alum, Harvard Law School
 Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="E105" t="inlineStr">
         <is>
           <t>2011 ACF Nationals Contributor
 2012 ACF Nationals Editor
 2013 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
         <is>
           <t>Bruce Lou</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>brucelou@gmail.com</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
         <is>
           <t>Alum, University of California, Berkeley</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t>2016 ACF Fall Editor
 2017 ACF Fall Editor
 2019 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
         <is>
           <t>Bryanna Shao</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>shao.bryanna@gmail.com</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
         <is>
           <t>Vanderbilt University</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>2020 ACF Winter Editor
 2022 ACF Fall Proofreader</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
         <is>
           <t>Carsten Gehring</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B108" t="inlineStr">
         <is>
           <t>octagonjoe@gmail.com</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
         <is>
           <t>Alum, Carleton College</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E108" t="inlineStr">
         <is>
           <t>2010 ACF Fall Editor
 2011 ACF Fall Head Editor
@@ -3739,91 +3768,91 @@
 2018 ACF Nationals Proofreader</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
         <is>
           <t>Chandler West</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>westchandler24@gmail.com</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
         <is>
           <t>M.Ed., Vanderbilt University
 Alum, Auburn University</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>2020 ACF Winter Editor
 2022 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
         <is>
           <t>Chris Ray</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>cwray30@gmail.com</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
         <is>
           <t>Ph.D. Candidate, The Ohio State University
 MA, University of Chicago
 Alum, University of Maryland</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
         <is>
           <t>David Hamilton</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>dhamiltn@gmail.com</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
         <is>
           <t>Fellow, Casualty Actuarial Society
 M.B.A, Elon University Love School of Business
 Alum, University of Maryland</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>1999 ACF Regionals Editor
 2000 ACF Nationals Editor
@@ -3831,63 +3860,63 @@
 Co-founder</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
         <is>
           <t>Dennis Jang</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>dennisjang@gmail.com</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
         <is>
           <t>Alum, Brown University</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>2007 ACF Fall Editor
 2009 ACF Winter Editor
 2010 ACF Winter Editor</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
         <is>
           <t>Dwight Wynne</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>dpwynne@gmail.com</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
         <is>
           <t>Ph.D. Candidate, Biomedical Engineering, University of California-Irvine
 Alum, University of California-Los Angeles</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E113" t="inlineStr">
         <is>
           <t>2009 ACF Nationals Editor
 2010 ACF Regionals Editor
@@ -3895,63 +3924,63 @@
 Designer of A-value qualification system</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
         <is>
           <t>Eddie Kim</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B114" t="inlineStr">
         <is>
           <t>eddie14dh@gmail.com</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
         <is>
           <t>SoCal Quizbowl</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="E114" t="inlineStr">
         <is>
           <t>2015 ACF Fall Editor
 2016 ACF Fall Editor
 2024 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
         <is>
           <t>Evan Adams</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>adamsej2@gmail.com</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
         <is>
           <t>Alum, University of Virginia Law School
 Alum, Virginia Commonwealth University</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E115" t="inlineStr">
         <is>
           <t>2009 ACF Fall Editor
 2010 ACF Fall Head Editor
@@ -3959,64 +3988,64 @@
 2017 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
         <is>
           <t>Evan Lynch</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B116" t="inlineStr">
         <is>
           <t>evanlynch@hotmail.co.uk</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
         <is>
           <t>Ph.D. Student, University of Southampton
 Alum, University of Cambridge</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="E116" t="inlineStr">
         <is>
           <t>2017 ACF Fall Editor
 2019 ACF Fall Logistics Support
 2020 ACF Regionals Logistics Support</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
         <is>
           <t>Gaurav Kandlikar</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B117" t="inlineStr">
         <is>
           <t>gaurav.kandlikar@gmail.com</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
         <is>
           <t>Ph.D. Student, UCLA
 Alum, University of Minnesota</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr">
+      <c r="E117" t="inlineStr">
         <is>
           <t>2011 ACF Fall Editor
 2014 ACF Fall Co-Head Editor
@@ -4024,31 +4053,31 @@
 2016 ACF Fall Head Editor</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
         <is>
           <t>Gautam Kandlikar</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>gautam.acf@gmail.com</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
         <is>
           <t>Alum, University of Minnesota</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr">
+      <c r="E118" t="inlineStr">
         <is>
           <t>2008 ACF Fall Editor
 2009 ACF Fall Head Editor
@@ -4056,216 +4085,216 @@
 2015-17, Treasurer</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
         <is>
           <t>Graham Reid</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B119" t="inlineStr">
         <is>
           <t>ghr180@gmail.com</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
         <is>
           <t>Alum, Kenyon College
 Ph.D., University of Maryland</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr">
+      <c r="E119" t="inlineStr">
         <is>
           <t>2019 ACF Regionals Editor
 2022 ACF Regionals Editor
 2023 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
         <is>
           <t>Guy Tabachnick</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B120" t="inlineStr">
         <is>
           <t>metsfan001@gmail.com</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
         <is>
           <t>Alum, Brown University</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr">
+      <c r="E120" t="inlineStr">
         <is>
           <t>2010 ACF Fall Editor
 2012 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
         <is>
           <t>Hasna Karim</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>hasna.saeeda.karim@gmail.com</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
         <is>
           <t>M.D. Candidate, Medical University of South Carolina
 Alum, Yale University</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
+      <c r="E121" t="inlineStr">
         <is>
           <t>2021 ACF Regionals Editor
 2023 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
         <is>
           <t>Jason Paik</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
+      <c r="B122" t="inlineStr">
         <is>
           <t>doctorandgeek@gmail.com</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
         <is>
           <t>MD/Ph.D., Cancer Biology, University of Alabama School of Medicine
 Alum, Washington University in St. Louis</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr">
+      <c r="E122" t="inlineStr">
         <is>
           <t>2004 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
         <is>
           <t>Jeff Hoppes</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B123" t="inlineStr">
         <is>
           <t>jeff.hoppes@gmail.com</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
         <is>
           <t>M.A., History, University of California, Berkeley
 Alum, Princeton University</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr">
+      <c r="E123" t="inlineStr">
         <is>
           <t>2005 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr"/>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
         <is>
           <t>Jennie Yang</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B124" t="inlineStr">
         <is>
           <t>yangjennie@gmail.com</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
         <is>
           <t>Alum, Stanford University</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E124" t="inlineStr">
         <is>
           <t>2017 ACF Fall Editor
 2019 ACF Regionals Editor
 2021 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
         <is>
           <t>Jerry Vinokurov</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
+      <c r="B125" t="inlineStr">
         <is>
           <t>grapesmoker@gmail.com</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
         <is>
           <t>Alum, University of California, Berkeley
 Ph.D., Brown University</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr">
+      <c r="E125" t="inlineStr">
         <is>
           <t>2007 ACF Regionals Editor
 2009 ACF Winter Head Editor
@@ -4277,31 +4306,31 @@
 2015–2017 ACF Nationals Tournament Director</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
         <is>
           <t>Jonathan Magin</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
+      <c r="B126" t="inlineStr">
         <is>
           <t>jonathan.magin@gmail.com</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
         <is>
           <t>Alum, University of Maryland</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr">
+      <c r="E126" t="inlineStr">
         <is>
           <t>2007 ACF Fall Editor
 2009 ACF Nationals Editor
@@ -4314,93 +4343,93 @@
 2021 ACF Online Moderator Training</t>
         </is>
       </c>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
         <is>
           <t>Jonathan Pinyan</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>pinyan@gmail.com</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
         <is>
           <t>Alum, Washington University in St. Louis</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr">
+      <c r="E127" t="inlineStr">
         <is>
           <t>2014 ACF Nationals Stats Director
 2015 ACF Nationals Stats Director
 2019 ACF Nationals Stats Director</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
         <is>
           <t>Margaret Tebbe</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>mtebbe@sas.upenn.edu</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
         <is>
           <t>Alum, University of Pennsylvania</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr">
+      <c r="E128" t="inlineStr">
         <is>
           <t>2019 ACF Nationals Host Logistics Contact
 2020-21, Site Coordinator</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
         <is>
           <t>Matt Jackson</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B129" t="inlineStr">
         <is>
           <t>mbjackson10@gmail.com</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
         <is>
           <t>M.S., University of Chicago
 Alum, Yale University</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr">
+      <c r="E129" t="inlineStr">
         <is>
           <t>2014 ACF Regionals Editor
 2015 ACF Nationals Assistant Tournament Director
@@ -4410,334 +4439,334 @@
 Lead writer, August 2016 ACF rules revision</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
         <is>
           <t>Matt Keller</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B130" t="inlineStr">
         <is>
           <t>mkvandy03@gmail.com</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
         <is>
           <t>Alum, Vanderbilt University</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr">
+      <c r="E130" t="inlineStr">
         <is>
           <t>2006 ACF Fall Editor
 2008 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
         <is>
           <t>Matt Lafer</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B131" t="inlineStr">
         <is>
           <t>matt.lafer@gmail.com</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
         <is>
           <t>Alum, University of Michigan</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr">
+      <c r="E131" t="inlineStr">
         <is>
           <t>2006 ACF Regionals Editor
 2008 ACF Nationals Editor
 2009 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
         <is>
           <t>Matt Reece</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
         <is>
           <t>Ph.D., Theoretical Physics, Cornell University
 Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E132" t="inlineStr">
         <is>
           <t>2010 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
         <is>
           <t>Max Schindler</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
+      <c r="B133" t="inlineStr">
         <is>
           <t>igoroogenflagenstein@gmail.com</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
         <is>
           <t>Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
+      <c r="E133" t="inlineStr">
         <is>
           <t>2014 ACF Fall Editor
 2016 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
         <is>
           <t>Mike Sorice</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B134" t="inlineStr">
         <is>
           <t>mike.sorice@gmail.com</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
         <is>
           <t>Alum, University of Illinois
 Alum, Eastern Illinois University</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr">
+      <c r="E134" t="inlineStr">
         <is>
           <t>2005 ACF Regionals Editor
 2006 ACF Regionals Head Editor
 2013 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
         <is>
           <t>Nathan Weiser</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>nlweiser@stanford.edu</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
         <is>
           <t>Alum, Stanford University</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>2015 ACF Fall Editor
 2017 ACF Regionals Editor
 2018 ACF Fall Head Editor</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
         <is>
           <t>Ned Tagtmeier</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B136" t="inlineStr">
         <is>
           <t>ned.tagtmeier@gmail.com</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
         <is>
           <t>University of Chicago</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr">
+      <c r="E136" t="inlineStr">
         <is>
           <t>2021 ACF Fall Editor
 2022 ACF Fall Editor</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
         <is>
           <t>Nitin Rao</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
+      <c r="B137" t="inlineStr">
         <is>
           <t>nitinsrao99@gmail.com</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
         <is>
           <t>J.D., Harvard Law School
 Alum, University of Pennsylvania</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr">
+      <c r="E137" t="inlineStr">
         <is>
           <t>2018 ACF Fall Editor
 2020 ACF Regionals Editor
 2021 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
         <is>
           <t>Paul Litvak</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B138" t="inlineStr">
         <is>
           <t>pmlitvak@gmail.com</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
         <is>
           <t>Ph.D., Behavioral Decision Making, Carnegie Mellon University
 Alum, University of Michigan</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr">
+      <c r="E138" t="inlineStr">
         <is>
           <t>2004 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
         <is>
           <t>Richard Yu</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
+      <c r="B139" t="inlineStr">
         <is>
           <t>th.richard.yu@gmail.com</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
         <is>
           <t>Alum, Washington University in St. Louis</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr">
+      <c r="E139" t="inlineStr">
         <is>
           <t>2014 ACF Fall Editor
 2015 ACF Fall Co-Head Editor
 2017 ACF Fall Editor</t>
         </is>
       </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
         <is>
           <t>Rob Carson</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
+      <c r="B140" t="inlineStr">
         <is>
           <t>rob.f.carson@gmail.com</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
         <is>
           <t>Alum, University of Minnesota</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr">
+      <c r="E140" t="inlineStr">
         <is>
           <t>2008 ACF Fall Editor
 2010 ACF Winter Editor
@@ -4750,31 +4779,31 @@
 2019 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F139" t="inlineStr"/>
-      <c r="G139" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
         <is>
           <t>Ryan Rosenberg</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
+      <c r="B141" t="inlineStr">
         <is>
           <t>ryanr345@gmail.com</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
         <is>
           <t>Alum, University of North Carolina at Chapel Hill</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr">
+      <c r="E141" t="inlineStr">
         <is>
           <t>2015 ACF Fall Editor
 2017 ACF Fall Editor
@@ -4785,32 +4814,32 @@
 2023 ACF Nationals Tournament Director</t>
         </is>
       </c>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
         <is>
           <t>Ryan Westbrook</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
+      <c r="B142" t="inlineStr">
         <is>
           <t>rwestb1212@gmail.com</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
         <is>
           <t>J.D., Wayne State University Law School
 Alum, University of Michigan</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr">
+      <c r="E142" t="inlineStr">
         <is>
           <t>2007 ACF Regionals Editor
 2008 ACF Nationals Editor
@@ -4822,32 +4851,32 @@
 2021 ACF Nationals Co-Head Editor</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
         <is>
           <t>Sam Luongo</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
+      <c r="B143" t="inlineStr">
         <is>
           <t>sangelo147@gmail.com</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
         <is>
           <t>Alum, Virginia Commonwealth University School of Education
 Alum, University of Virginia</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr">
+      <c r="E143" t="inlineStr">
         <is>
           <t>2011 ACF Fall Editor
 2015 ACF Regionals Editor and Logistics Coordinator
@@ -4856,64 +4885,64 @@
 2018 ACF Nationals Tournament Director</t>
         </is>
       </c>
-      <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
         <is>
           <t>Seth Teitler</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
+      <c r="B144" t="inlineStr">
         <is>
           <t>satelite@gmail.com</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
         <is>
           <t>Ph.D., Astrophysics, University of Chicago
 Alum, University of California, Berkeley</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr">
+      <c r="E144" t="inlineStr">
         <is>
           <t>2005 ACF Fall Editor
 2007 ACF Regionals Head Editor
 2009 ACF Fall Advisor</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
         <is>
           <t>Stephen Eltinge</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
+      <c r="B145" t="inlineStr">
         <is>
           <t>stepheneltinge@gmail.com</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
         <is>
           <t>Ph.D., Yale University
 Alum, MIT</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr">
+      <c r="E145" t="inlineStr">
         <is>
           <t>2013 ACF Fall Editor
 2014-17, Communications Officer
@@ -4922,32 +4951,32 @@
 2022 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
         <is>
           <t>Stephen Liu</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
+      <c r="B146" t="inlineStr">
         <is>
           <t>stephen.jhliu@gmail.com</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
         <is>
           <t>J.D., Stanford Law School
 Alum, Harvard University</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr">
+      <c r="E146" t="inlineStr">
         <is>
           <t>2012 ACF Fall Editor
 2013 ACF Fall Head Editor
@@ -4958,92 +4987,92 @@
 2024 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
         <is>
           <t>Steven Liu</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
+      <c r="B147" t="inlineStr">
         <is>
           <t>sirmrguy1153@gmail.com</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
         <is>
           <t>Alum, MIT</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr">
+      <c r="E147" t="inlineStr">
         <is>
           <t>2021 ACF Winter Editor
 2022 ACF Fall Co-Head Editor</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
         <is>
           <t>Subash Maddipoti</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
+      <c r="B148" t="inlineStr">
         <is>
           <t>suby10@gmail.com</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
         <is>
           <t>Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr">
+      <c r="E148" t="inlineStr">
         <is>
           <t>2001 ACF Nationals Editor
 2004 ACF Fall Head Editor</t>
         </is>
       </c>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
         <is>
           <t>Susan Ferrari</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
+      <c r="B149" t="inlineStr">
         <is>
           <t>srferrar@gmail.com</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
         <is>
           <t>Ph.D., Cancer Biology, University of Chicago
 Alum, University of Chicago</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr">
+      <c r="E149" t="inlineStr">
         <is>
           <t>2010 ACF Nationals Editor
 2011-14, Communications Officer
@@ -5051,31 +5080,31 @@
 2012 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
         <is>
           <t>Ted Gioia</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B150" t="inlineStr">
         <is>
           <t>tgioia4@gmail.com</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
         <is>
           <t>Alum, Harvard University</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E150" t="inlineStr">
         <is>
           <t>2008 ACF Fall Editor
 2010 ACF Regionals Editor
@@ -5083,94 +5112,94 @@
 2014 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
         <is>
           <t>Theresa Nyowheoma</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B151" t="inlineStr">
         <is>
           <t>theresa.nyowheoma@outlook.com</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
         <is>
           <t>Alum, New York University</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr">
+      <c r="E151" t="inlineStr">
         <is>
           <t>2020 ACF Fall Tournament Director
 2021-22, Site Coordinator
 2021 ACF Regionals Tournament Director</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
         <is>
           <t>Tommy Casalaspi</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B152" t="inlineStr">
         <is>
           <t>casalaspi@g.harvard.edu</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
         <is>
           <t>Ph.D. Student, Harvard University
 University of Virginia</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E152" t="inlineStr">
         <is>
           <t>2015 ACF Regionals Editor
 2017 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
         <is>
           <t>Trevor Davis</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B153" t="inlineStr">
         <is>
           <t>TheBokonon@gmail.com</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
         <is>
           <t>Graduate Student, University of Alberta
 Alum, Carnegie Mellon University</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr">
+      <c r="E153" t="inlineStr">
         <is>
           <t>2008 ACF Fall Editor
 2010 ACF Winter Editor
@@ -5178,145 +5207,145 @@
 2015 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
         <is>
           <t>Trygve Meade</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr"/>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
         <is>
           <t>Alum, Southern Illinois University Law School
 Alum, University of Illinois</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr">
+      <c r="E154" t="inlineStr">
         <is>
           <t>2009 ACF Winter Editor
 2010 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>Wesley Matthews</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr"/>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>Alum, Indiana University</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr">
-        <is>
-          <t>2008 ACF Nationals Editor</t>
-        </is>
-      </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
+          <t>Wesley Matthews</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Alum, Indiana University</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2008 ACF Nationals Editor</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
           <t>Will Butler</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B156" t="inlineStr">
         <is>
           <t>tachyonwill@gmail.com</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
         <is>
           <t>Ph.D. Student, Biology, Georgia Tech
 Alum, University of Virginia</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr">
+      <c r="E156" t="inlineStr">
         <is>
           <t>2010 ACF Fall Editor
 2012 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
         <is>
           <t>Will Holub-Moorman</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B157" t="inlineStr">
         <is>
           <t>holubmoorman@gmail.com</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
         <is>
           <t>Alum, Harvard University</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr">
+      <c r="E157" t="inlineStr">
         <is>
           <t>2018 ACF Regionals Editor
 2019 ACF Regionals Editor</t>
         </is>
       </c>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
         <is>
           <t>Will Nediger</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B158" t="inlineStr">
         <is>
           <t>wnediger@umich.edu</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
         <is>
           <t>Ph.D., University of Michigan
 Alum, University of Western Ontario</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr">
+      <c r="E158" t="inlineStr">
         <is>
           <t>2009 ACF Fall Editor
 2014 ACF Regionals Editor
@@ -5324,97 +5353,76 @@
 2023 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
         <is>
           <t>William Golden</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B159" t="inlineStr">
         <is>
           <t>williamgolden14@gmail.com</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
         <is>
           <t>Alum, University of Texas at Austin</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr">
+      <c r="E159" t="inlineStr">
         <is>
           <t>2020 ACF Winter Head Editor
 2023 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
         <is>
           <t>Zeke Berdichevsky</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B160" t="inlineStr">
         <is>
           <t>eberdich@gmail.com</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>emeritus</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>emeritus</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
         <is>
           <t>J.D., George Washington University Law School
 M.A., Ph.D. Candidate (ABD), English Literature, University of Michigan
 Alum, University of Maryland</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr">
+      <c r="E160" t="inlineStr">
         <is>
           <t>2002 ACF Regionals Head Editor
 2004 ACF Nationals Head Editor
 2010 ACF Nationals Head Editor</t>
         </is>
       </c>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>Auroni Gupta</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr"/>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>former</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr"/>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>2019 ACF Nationals Head Editor</t>
-        </is>
-      </c>
       <c r="F160" t="inlineStr"/>
       <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Chris Romero</t>
+          <t>Auroni Gupta</t>
         </is>
       </c>
       <c r="B161" t="inlineStr"/>
@@ -5424,14 +5432,18 @@
         </is>
       </c>
       <c r="D161" t="inlineStr"/>
-      <c r="E161" t="inlineStr"/>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2019 ACF Nationals Head Editor</t>
+        </is>
+      </c>
       <c r="F161" t="inlineStr"/>
       <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Eric Kwartler</t>
+          <t>Chris Romero</t>
         </is>
       </c>
       <c r="B162" t="inlineStr"/>
@@ -5441,61 +5453,78 @@
         </is>
       </c>
       <c r="D162" t="inlineStr"/>
-      <c r="E162" t="inlineStr">
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Eric Kwartler</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr"/>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>former</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr">
         <is>
           <t>2007 ACF Fall Head Editor?
 2006 ACF Fall Head Editor?
 2005 ACF Fall Head Editor?</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
         <is>
           <t>Evan Knox</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B164" t="inlineStr">
         <is>
           <t>evanknoxgrad@gmail.com</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
+      <c r="C164" t="inlineStr">
         <is>
           <t>former</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr"/>
-      <c r="E163" t="inlineStr">
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr">
         <is>
           <t>2022 ACF Fall Editor
 2023 ACF Fall Editor
 2023 ACF Winter Editor</t>
         </is>
       </c>
-      <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
         <is>
           <t>Ike Jose</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B165" t="inlineStr">
         <is>
           <t>sephiroth0kouko@gmail.com</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C165" t="inlineStr">
         <is>
           <t>former</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr"/>
-      <c r="E164" t="inlineStr">
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr">
         <is>
           <t>2019 ACF Nationals Editor
 2017 ACF Nationals Editor
@@ -5503,43 +5532,18 @@
 2015 ACF Nationals Editor</t>
         </is>
       </c>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>Jack Mehr</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>mehrj14@gmail.com</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>former</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr"/>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>2021 ACF Nationals Editor</t>
-        </is>
-      </c>
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Justin Jasperse</t>
+          <t>Jack Mehr</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>justinjasperse2022@u.northwestern.edu</t>
+          <t>mehrj14@gmail.com</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -5550,7 +5554,7 @@
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>2021 ACF Nationals Host Logistics Contact</t>
+          <t>2021 ACF Nationals Editor</t>
         </is>
       </c>
       <c r="F166" t="inlineStr"/>
@@ -5559,12 +5563,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Karan Gurazada</t>
+          <t>Justin Jasperse</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>karangurazada@gmail.com</t>
+          <t>justinjasperse2022@u.northwestern.edu</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -5575,7 +5579,7 @@
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2021 ACF Fall Editor</t>
+          <t>2021 ACF Nationals Host Logistics Contact</t>
         </is>
       </c>
       <c r="F167" t="inlineStr"/>
@@ -5584,10 +5588,14 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Kelly McKenzie</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr"/>
+          <t>Karan Gurazada</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>karangurazada@gmail.com</t>
+        </is>
+      </c>
       <c r="C168" t="inlineStr">
         <is>
           <t>former</t>
@@ -5595,66 +5603,87 @@
       </c>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
+        <is>
+          <t>2021 ACF Fall Editor</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Kelly McKenzie</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr"/>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>former</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
         <is>
           <t>2003 ACF Fall Head Editor
 2002 ACF Fall Head Editor
 2001 ACF Fall Head Editor</t>
         </is>
       </c>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>Kevin Park</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>kevinpark27@gmail.com</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>former</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>Pomona College</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>2023 ACF Regionals Editor</t>
-        </is>
-      </c>
       <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>2022-23</t>
-        </is>
-      </c>
+      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
+          <t>Kevin Park</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>kevinpark27@gmail.com</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>former</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Pomona College</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2023 ACF Regionals Editor</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>2022-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
           <t>Matt Weiner</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B171" t="inlineStr">
         <is>
           <t>mattweiner.vcu@gmail.com</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C171" t="inlineStr">
         <is>
           <t>former</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr"/>
-      <c r="E170" t="inlineStr">
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr">
         <is>
           <t>2011 ACF Regionals Editor
 2008 ACF Regionals Head Editor
@@ -5664,43 +5693,18 @@
 2005 ACF Fall Editor</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>Matthew Lehmann</t>
-        </is>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>matthewlehmann18@gmail.com</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>former</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr"/>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>2020 ACF Fall Editor and Oversight</t>
-        </is>
-      </c>
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Mia McGill</t>
+          <t>Matthew Lehmann</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>miamc.qb@gmail.com</t>
+          <t>matthewlehmann18@gmail.com</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -5711,47 +5715,47 @@
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
+          <t>2020 ACF Fall Editor and Oversight</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Mia McGill</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>miamc.qb@gmail.com</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>former</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr">
+        <is>
           <t>2022-23, Communications Officer
 2022 ACF Nationals Logistics Coordinator</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>Natan Holtzman</t>
-        </is>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>natan.holtzman@gmail.com</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>former</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr"/>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>2021 ACF Regionals Editor</t>
-        </is>
-      </c>
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Olivia Murton</t>
+          <t>Natan Holtzman</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>omurton@gmail.com</t>
+          <t>natan.holtzman@gmail.com</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -5761,6 +5765,31 @@
       </c>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
+        <is>
+          <t>2021 ACF Regionals Editor</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Olivia Murton</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>omurton@gmail.com</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>former</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr"/>
+      <c r="E175" t="inlineStr">
         <is>
           <t>2022 ACF Nationals Proofreader
 Communications Officer, 2021-22
@@ -5769,43 +5798,18 @@
 2021 ACF Regionals Logistics Support &amp; Proofreader</t>
         </is>
       </c>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>Angela Lin</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>ahlin@berkeley.edu</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>nonmember</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr"/>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>2021 ACF Winter Editor</t>
-        </is>
-      </c>
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Daniel Ma</t>
+          <t>Angela Lin</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>danielma4114@gmail.com</t>
+          <t>ahlin@berkeley.edu</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -5813,14 +5817,10 @@
           <t>nonmember</t>
         </is>
       </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Alum, Yale University</t>
-        </is>
-      </c>
+      <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>2022 ACF Fall Editor</t>
+          <t>2021 ACF Winter Editor</t>
         </is>
       </c>
       <c r="F176" t="inlineStr"/>

</xml_diff>

<commit_message>
Collection of minor site updates
</commit_message>
<xml_diff>
--- a/about/members.xlsx
+++ b/about/members.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G179"/>
+  <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,11 +445,6 @@
       <c r="F1" t="inlineStr">
         <is>
           <t>Skills</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Last Activity</t>
         </is>
       </c>
     </row>
@@ -485,7 +480,6 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -516,7 +510,6 @@
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -547,7 +540,6 @@
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -577,7 +569,6 @@
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -612,7 +603,6 @@
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -649,7 +639,6 @@
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -685,7 +674,6 @@
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -716,7 +704,6 @@
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -746,7 +733,6 @@
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -777,7 +763,6 @@
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -808,7 +793,6 @@
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -835,11 +819,11 @@
         <is>
           <t>2022 ACF Nationals Assistant Tournament Director
 2023-24, Communications Officer
-2023 ACF Nationals Liveblogging/On-site Communications Coordinator</t>
+2023 ACF Nationals Liveblog Coordinator
+2023 ACF Nationals On-site Communications Coordinator</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -870,7 +854,6 @@
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -903,7 +886,6 @@
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -940,7 +922,6 @@
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -971,7 +952,6 @@
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1002,7 +982,6 @@
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1034,7 +1013,6 @@
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1065,7 +1043,6 @@
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1095,7 +1072,6 @@
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1121,7 +1097,6 @@
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1154,7 +1129,6 @@
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1193,7 +1167,6 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1226,7 +1199,6 @@
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1262,7 +1234,6 @@
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1291,7 +1262,6 @@
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1328,7 +1298,6 @@
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1361,7 +1330,6 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1394,7 +1362,6 @@
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1427,7 +1394,6 @@
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1464,7 +1430,6 @@
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1490,7 +1455,6 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1523,7 +1487,6 @@
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1558,7 +1521,6 @@
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1592,7 +1554,6 @@
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1612,7 +1573,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ph.D. Student, Penn State University
+          <t>Alum, Penn State University
 Alum, University of Illinois</t>
         </is>
       </c>
@@ -1623,7 +1584,6 @@
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1643,7 +1603,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ph.D. Student, Stanford University</t>
+          <t>Ph.D., Stanford University</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1655,7 +1615,6 @@
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1691,7 +1650,6 @@
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1724,7 +1682,6 @@
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1754,7 +1711,6 @@
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1785,7 +1741,6 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1817,7 +1772,6 @@
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1850,7 +1804,6 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1880,7 +1833,6 @@
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1911,7 +1863,6 @@
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1942,7 +1893,6 @@
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1972,7 +1922,6 @@
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2002,7 +1951,6 @@
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2022,7 +1970,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Ph.D. Student, Northwestern University
+          <t>Ph.D., Northwestern University
 Alum, University of Toronto</t>
         </is>
       </c>
@@ -2036,7 +1984,6 @@
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2066,7 +2013,6 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2096,7 +2042,6 @@
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2133,7 +2078,6 @@
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2159,7 +2103,6 @@
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2189,7 +2132,6 @@
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2220,7 +2162,6 @@
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2246,7 +2187,6 @@
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2277,7 +2217,6 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2306,7 +2245,6 @@
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2335,7 +2273,6 @@
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2365,7 +2302,6 @@
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2394,7 +2330,6 @@
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2423,7 +2358,6 @@
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2452,7 +2386,6 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2481,7 +2414,6 @@
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2510,7 +2442,6 @@
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2539,7 +2470,6 @@
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2564,7 +2494,6 @@
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2589,7 +2518,6 @@
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2618,7 +2546,6 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2647,7 +2574,6 @@
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2676,7 +2602,6 @@
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2705,7 +2630,6 @@
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2735,7 +2659,6 @@
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2765,7 +2688,6 @@
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2795,7 +2717,6 @@
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2824,7 +2745,6 @@
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2853,7 +2773,6 @@
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2882,7 +2801,6 @@
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2907,7 +2825,6 @@
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2936,7 +2853,6 @@
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2965,7 +2881,6 @@
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2994,7 +2909,6 @@
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3024,7 +2938,6 @@
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3055,7 +2968,6 @@
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3084,7 +2996,6 @@
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3113,7 +3024,6 @@
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3142,7 +3052,6 @@
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3171,7 +3080,6 @@
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3200,7 +3108,6 @@
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3232,7 +3139,6 @@
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3261,7 +3167,6 @@
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3286,7 +3191,6 @@
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3315,7 +3219,6 @@
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3348,7 +3251,6 @@
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3380,7 +3282,6 @@
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3401,7 +3302,7 @@
       <c r="D97" t="inlineStr">
         <is>
           <t>J.D., George Washington University Law School
-M.A., Ph.D. Candidate (ABD), English Literature, University of Michigan
+M.A., Ph.D. Candidate (ABD), University of Michigan
 Alum, University of Maryland</t>
         </is>
       </c>
@@ -3413,7 +3314,6 @@
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3447,7 +3347,6 @@
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3478,7 +3377,6 @@
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3515,7 +3413,6 @@
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3546,7 +3443,6 @@
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3581,7 +3477,6 @@
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3614,7 +3509,6 @@
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3648,7 +3542,6 @@
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3680,7 +3573,6 @@
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3713,7 +3605,6 @@
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3746,7 +3637,6 @@
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3778,7 +3668,6 @@
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3808,7 +3697,6 @@
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3842,7 +3730,6 @@
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3872,7 +3759,6 @@
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3902,7 +3788,6 @@
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3937,7 +3822,6 @@
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3968,7 +3852,6 @@
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4001,7 +3884,6 @@
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4033,7 +3915,6 @@
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4064,7 +3945,6 @@
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4094,7 +3974,6 @@
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4125,7 +4004,6 @@
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4156,7 +4034,6 @@
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4176,7 +4053,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Ph.D., Behavioral Decision Making, Carnegie Mellon University
+          <t>Ph.D., Carnegie Mellon University
 Alum, University of Michigan</t>
         </is>
       </c>
@@ -4186,7 +4063,6 @@
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4222,7 +4098,6 @@
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4252,7 +4127,6 @@
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4283,7 +4157,6 @@
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4317,7 +4190,6 @@
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4349,7 +4221,6 @@
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4379,7 +4250,6 @@
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4416,7 +4286,6 @@
         </is>
       </c>
       <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4441,7 +4310,6 @@
         </is>
       </c>
       <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4468,7 +4336,6 @@
         </is>
       </c>
       <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4498,7 +4365,6 @@
         </is>
       </c>
       <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4529,7 +4395,6 @@
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4562,7 +4427,6 @@
         </is>
       </c>
       <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4593,7 +4457,6 @@
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4613,7 +4476,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>MD/Ph.D., Cancer Biology, University of Alabama School of Medicine
+          <t>MD/Ph.D., University of Alabama School of Medicine
 Alum, Washington University in St. Louis</t>
         </is>
       </c>
@@ -4623,7 +4486,6 @@
         </is>
       </c>
       <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4654,7 +4516,6 @@
         </is>
       </c>
       <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4686,7 +4547,6 @@
         </is>
       </c>
       <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4713,7 +4573,6 @@
       </c>
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4739,7 +4598,6 @@
         </is>
       </c>
       <c r="F139" t="inlineStr"/>
-      <c r="G139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4771,7 +4629,6 @@
         </is>
       </c>
       <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4791,7 +4648,8 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Alum, University of North Carolina at Chapel Hill</t>
+          <t>New York University
+Alum, University of North Carolina at Chapel Hill</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -4806,7 +4664,6 @@
         </is>
       </c>
       <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4836,7 +4693,6 @@
         </is>
       </c>
       <c r="F142" t="inlineStr"/>
-      <c r="G142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4866,7 +4722,6 @@
         </is>
       </c>
       <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4900,7 +4755,6 @@
         </is>
       </c>
       <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4932,7 +4786,6 @@
         </is>
       </c>
       <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4965,7 +4818,6 @@
         </is>
       </c>
       <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4995,7 +4847,6 @@
         </is>
       </c>
       <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5025,7 +4876,6 @@
         </is>
       </c>
       <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5055,7 +4905,6 @@
         </is>
       </c>
       <c r="F149" t="inlineStr"/>
-      <c r="G149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5087,7 +4936,6 @@
         </is>
       </c>
       <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5124,7 +4972,6 @@
         </is>
       </c>
       <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5156,7 +5003,6 @@
         </is>
       </c>
       <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5187,7 +5033,6 @@
         </is>
       </c>
       <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5218,7 +5063,6 @@
         </is>
       </c>
       <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5255,7 +5099,6 @@
         </is>
       </c>
       <c r="F155" t="inlineStr"/>
-      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5275,7 +5118,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Ph.D. Candidate, Biomedical Engineering, University of California-Irvine
+          <t>Ph.D. Candidate, University of California-Irvine
 Alum, University of California-Los Angeles</t>
         </is>
       </c>
@@ -5288,7 +5131,6 @@
         </is>
       </c>
       <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5319,7 +5161,6 @@
         </is>
       </c>
       <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -5350,7 +5191,6 @@
         </is>
       </c>
       <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5387,7 +5227,6 @@
         </is>
       </c>
       <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5418,7 +5257,6 @@
         </is>
       </c>
       <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -5439,7 +5277,6 @@
         </is>
       </c>
       <c r="F161" t="inlineStr"/>
-      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -5464,7 +5301,6 @@
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -5489,7 +5325,6 @@
         </is>
       </c>
       <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -5514,7 +5349,6 @@
         </is>
       </c>
       <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -5542,7 +5376,6 @@
         </is>
       </c>
       <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -5569,7 +5402,6 @@
         </is>
       </c>
       <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -5592,7 +5424,6 @@
         </is>
       </c>
       <c r="F167" t="inlineStr"/>
-      <c r="G167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -5617,7 +5448,6 @@
         </is>
       </c>
       <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5643,7 +5473,6 @@
         </is>
       </c>
       <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5666,7 +5495,6 @@
         </is>
       </c>
       <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5691,7 +5519,6 @@
         </is>
       </c>
       <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5720,7 +5547,6 @@
         </is>
       </c>
       <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5749,11 +5575,6 @@
         </is>
       </c>
       <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>2022-23</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5770,7 +5591,6 @@
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5800,7 +5620,6 @@
         </is>
       </c>
       <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5825,7 +5644,6 @@
         </is>
       </c>
       <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5850,7 +5668,6 @@
         </is>
       </c>
       <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -5875,7 +5692,6 @@
         </is>
       </c>
       <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -5900,7 +5716,6 @@
         </is>
       </c>
       <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>